<commit_message>
Small changes in diffussion mechanism, cleaning residual files
</commit_message>
<xml_diff>
--- a/currentEMCHA_last.xlsx
+++ b/currentEMCHA_last.xlsx
@@ -1,21 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://tcdud-my.sharepoint.com/personal/gimenezs_tcd_ie/Documents/Projects/eMCHA-STOSS/CISS_2006_last_gerliz/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://tcdud-my.sharepoint.com/personal/gimenezs_tcd_ie/Documents/Projects/eMCHA-STOSS/kMC4eMCHA/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{5E65ED4A-7381-4778-9827-E29241BCD971}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="65" documentId="8_{5E65ED4A-7381-4778-9827-E29241BCD971}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6BCCE09A-F3E1-486E-91A6-8CB1B22A24DE}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{837A7F63-7E9C-44D6-B236-481921DD8ADC}"/>
+    <workbookView xWindow="390" yWindow="390" windowWidth="21600" windowHeight="12645" xr2:uid="{837A7F63-7E9C-44D6-B236-481921DD8ADC}"/>
+    <workbookView xWindow="1980" yWindow="-15375" windowWidth="24405" windowHeight="13425" xr2:uid="{C5DCD740-E4AD-43D4-B043-660A1F5AE3AA}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191029" fullCalcOnLoad="1"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -98,9 +99,6 @@
     <t>V=-0.15</t>
   </si>
   <si>
-    <t>V=0.0765</t>
-  </si>
-  <si>
     <t>deltaR'</t>
   </si>
   <si>
@@ -110,7 +108,10 @@
     <t>gamma</t>
   </si>
   <si>
-    <t>V=-0.0765</t>
+    <t>V=0.0755</t>
+  </si>
+  <si>
+    <t>V=-0.0755</t>
   </si>
 </sst>
 </file>
@@ -325,7 +326,7 @@
   </cellStyleXfs>
   <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -379,6 +380,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -701,8 +706,9 @@
   <dimension ref="A1:L121"/>
   <sheetFormatPr defaultRowHeight="12.75"/>
   <cols>
-    <col min="1" max="2" width="18.7109375" style="2" customWidth="1"/>
-    <col min="3" max="3" width="14.5703125" style="2" customWidth="1"/>
+    <col min="1" max="1" width="10.140625" style="2" customWidth="1"/>
+    <col min="2" max="2" width="13.140625" style="2" customWidth="1"/>
+    <col min="3" max="3" width="13.5703125" style="2" customWidth="1"/>
     <col min="4" max="4" width="15" style="2" customWidth="1"/>
     <col min="5" max="5" width="12.140625" style="2" customWidth="1"/>
     <col min="6" max="6" width="18.42578125" style="2" customWidth="1"/>
@@ -743,7 +749,7 @@
     </row>
     <row r="5" spans="1:5">
       <c r="A5" s="2">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="B5" s="2">
         <v>0</v>
@@ -815,8 +821,7 @@
     </row>
     <row r="15" spans="1:5" customFormat="1">
       <c r="B15" s="2">
-        <f t="shared" si="0"/>
-        <v>0.99999999999999989</v>
+        <v>50</v>
       </c>
     </row>
     <row r="16" spans="1:5" customFormat="1"/>
@@ -893,7 +898,7 @@
     <row r="29" spans="1:4" customFormat="1">
       <c r="A29">
         <f t="shared" si="1"/>
-        <v>0.6724930681007999</v>
+        <v>33.62465340504</v>
       </c>
     </row>
     <row r="30" spans="1:4" customFormat="1"/>
@@ -969,7 +974,7 @@
     <row r="42" spans="1:3" customFormat="1">
       <c r="A42">
         <f t="shared" si="2"/>
-        <v>1.3449861362015998</v>
+        <v>67.24930681008</v>
       </c>
     </row>
     <row r="43" spans="1:3" customFormat="1"/>
@@ -996,32 +1001,32 @@
       <c r="A47" s="2"/>
       <c r="B47">
         <f t="shared" si="3"/>
-        <v>0.50420298267682562</v>
+        <v>0.5168059934641247</v>
       </c>
       <c r="C47">
         <f t="shared" si="4"/>
-        <v>0.49579701732317438</v>
+        <v>0.48319400653587524</v>
       </c>
     </row>
     <row r="48" spans="1:3" customFormat="1">
       <c r="B48">
         <f t="shared" si="3"/>
-        <v>0.50840537142797515</v>
+        <v>0.53357405611241004</v>
       </c>
       <c r="C48">
         <f t="shared" si="4"/>
-        <v>0.49159462857202485</v>
+        <v>0.46642594388759007</v>
       </c>
     </row>
     <row r="49" spans="1:7">
       <c r="A49"/>
       <c r="B49">
         <f t="shared" si="3"/>
-        <v>0.5126065726634369</v>
+        <v>0.5502665987944777</v>
       </c>
       <c r="C49">
         <f t="shared" si="4"/>
-        <v>0.4873934273365631</v>
+        <v>0.4497334012055223</v>
       </c>
       <c r="D49"/>
       <c r="E49"/>
@@ -1031,11 +1036,11 @@
       <c r="A50"/>
       <c r="B50">
         <f t="shared" si="3"/>
-        <v>0.5168059934641247</v>
+        <v>0.56684670917173086</v>
       </c>
       <c r="C50">
         <f t="shared" si="4"/>
-        <v>0.48319400653587524</v>
+        <v>0.4331532908282692</v>
       </c>
       <c r="D50"/>
       <c r="E50"/>
@@ -1045,11 +1050,11 @@
       <c r="A51"/>
       <c r="B51">
         <f t="shared" si="3"/>
-        <v>0.5210030419163344</v>
+        <v>0.58327847403800337</v>
       </c>
       <c r="C51">
         <f t="shared" si="4"/>
-        <v>0.47899695808366566</v>
+        <v>0.41672152596199674</v>
       </c>
       <c r="D51"/>
       <c r="E51"/>
@@ -1059,11 +1064,11 @@
       <c r="A52"/>
       <c r="B52">
         <f t="shared" si="3"/>
-        <v>0.52519712744499347</v>
+        <v>0.59952728292269697</v>
       </c>
       <c r="C52">
         <f t="shared" si="4"/>
-        <v>0.47480287255500653</v>
+        <v>0.40047271707730309</v>
       </c>
       <c r="D52"/>
       <c r="E52"/>
@@ -1073,11 +1078,11 @@
       <c r="A53"/>
       <c r="B53">
         <f t="shared" si="3"/>
-        <v>0.529387661145308</v>
+        <v>0.61556010768097025</v>
       </c>
       <c r="C53">
         <f t="shared" si="4"/>
-        <v>0.47061233885469206</v>
+        <v>0.3844398923190297</v>
       </c>
       <c r="D53"/>
       <c r="E53"/>
@@ -1087,11 +1092,11 @@
       <c r="A54"/>
       <c r="B54">
         <f t="shared" si="3"/>
-        <v>0.53357405611241004</v>
+        <v>0.63134575352492717</v>
       </c>
       <c r="C54">
         <f t="shared" si="4"/>
-        <v>0.46642594388759007</v>
+        <v>0.36865424647507272</v>
       </c>
       <c r="D54"/>
       <c r="E54"/>
@@ -1101,11 +1106,11 @@
       <c r="A55"/>
       <c r="B55">
         <f t="shared" si="3"/>
-        <v>0.53775572776861602</v>
+        <v>0.64685507781690388</v>
       </c>
       <c r="C55">
         <f t="shared" si="4"/>
-        <v>0.46224427223138398</v>
+        <v>0.35314492218309612</v>
       </c>
       <c r="D55"/>
       <c r="E55"/>
@@ -1115,11 +1120,11 @@
       <c r="A56"/>
       <c r="B56">
         <f t="shared" si="3"/>
-        <v>0.54193209418791022</v>
+        <v>0.99999999999999756</v>
       </c>
       <c r="C56">
         <f t="shared" si="4"/>
-        <v>0.45806790581208973</v>
+        <v>2.4945865146310072E-15</v>
       </c>
       <c r="D56"/>
       <c r="E56"/>
@@ -1212,11 +1217,11 @@
     <row r="63" spans="1:7">
       <c r="B63" s="5">
         <f t="shared" si="5"/>
-        <v>0.49579701732317438</v>
+        <v>0.48319400653587524</v>
       </c>
       <c r="C63" s="5">
         <f t="shared" si="6"/>
-        <v>0.50420298267682562</v>
+        <v>0.5168059934641247</v>
       </c>
       <c r="D63" s="5">
         <f t="shared" ref="D63:D72" si="9">D62</f>
@@ -1228,21 +1233,21 @@
       </c>
       <c r="F63" s="6">
         <f t="shared" si="7"/>
-        <v>0.34384609175193992</v>
+        <v>0.34570219260383284</v>
       </c>
       <c r="G63">
         <f t="shared" si="8"/>
-        <v>0.43624168951791997</v>
+        <v>0.433899475355358</v>
       </c>
     </row>
     <row r="64" spans="1:7">
       <c r="B64" s="5">
         <f t="shared" si="5"/>
-        <v>0.49159462857202485</v>
+        <v>0.46642594388759007</v>
       </c>
       <c r="C64" s="5">
         <f t="shared" si="6"/>
-        <v>0.50840537142797515</v>
+        <v>0.53357405611240993</v>
       </c>
       <c r="D64" s="5">
         <f t="shared" si="9"/>
@@ -1254,21 +1259,21 @@
       </c>
       <c r="F64" s="6">
         <f t="shared" si="7"/>
-        <v>0.34446499603383218</v>
+        <v>0.34817169896952149</v>
       </c>
       <c r="G64">
         <f t="shared" si="8"/>
-        <v>0.43545788897884852</v>
+        <v>0.43082192046037265</v>
       </c>
     </row>
     <row r="65" spans="1:9">
       <c r="B65" s="5">
         <f t="shared" si="5"/>
-        <v>0.4873934273365631</v>
+        <v>0.4497334012055223</v>
       </c>
       <c r="C65" s="5">
         <f t="shared" si="6"/>
-        <v>0.5126065726634369</v>
+        <v>0.5502665987944777</v>
       </c>
       <c r="D65" s="5">
         <f t="shared" si="9"/>
@@ -1280,21 +1285,21 @@
       </c>
       <c r="F65" s="6">
         <f t="shared" si="7"/>
-        <v>0.34508372542506405</v>
+        <v>0.35063008317749744</v>
       </c>
       <c r="G65">
         <f t="shared" si="8"/>
-        <v>0.43467712021259297</v>
+        <v>0.42780128459219047</v>
       </c>
     </row>
     <row r="66" spans="1:9">
       <c r="B66" s="5">
         <f t="shared" si="5"/>
-        <v>0.48319400653587524</v>
+        <v>0.4331532908282692</v>
       </c>
       <c r="C66" s="5">
         <f t="shared" si="6"/>
-        <v>0.5168059934641247</v>
+        <v>0.56684670917173086</v>
       </c>
       <c r="D66" s="5">
         <f t="shared" si="9"/>
@@ -1306,21 +1311,21 @@
       </c>
       <c r="F66" s="6">
         <f t="shared" si="7"/>
-        <v>0.34570219260383284</v>
+        <v>0.35307190898524121</v>
       </c>
       <c r="G66">
         <f t="shared" si="8"/>
-        <v>0.433899475355358</v>
+        <v>0.42484263455315036</v>
       </c>
     </row>
     <row r="67" spans="1:9">
       <c r="B67" s="5">
         <f t="shared" si="5"/>
-        <v>0.47899695808366566</v>
+        <v>0.41672152596199674</v>
       </c>
       <c r="C67" s="5">
         <f t="shared" si="6"/>
-        <v>0.52100304191633429</v>
+        <v>0.58327847403800326</v>
       </c>
       <c r="D67" s="5">
         <f t="shared" si="9"/>
@@ -1332,21 +1337,21 @@
       </c>
       <c r="F67" s="6">
         <f t="shared" si="7"/>
-        <v>0.34632031039640299</v>
+        <v>0.35549188729686254</v>
       </c>
       <c r="G67">
         <f t="shared" si="8"/>
-        <v>0.43312504492822823</v>
+        <v>0.42195055741100129</v>
       </c>
     </row>
     <row r="68" spans="1:9">
       <c r="B68" s="5">
         <f t="shared" si="5"/>
-        <v>0.47480287255500653</v>
+        <v>0.40047271707730309</v>
       </c>
       <c r="C68" s="5">
         <f t="shared" si="6"/>
-        <v>0.52519712744499347</v>
+        <v>0.59952728292269697</v>
       </c>
       <c r="D68" s="5">
         <f t="shared" si="9"/>
@@ -1358,21 +1363,21 @@
       </c>
       <c r="F68" s="6">
         <f t="shared" si="7"/>
-        <v>0.34693799182618495</v>
+        <v>0.35788492087607049</v>
       </c>
       <c r="G68">
         <f t="shared" si="8"/>
-        <v>0.43235391780082016</v>
+        <v>0.41912914249869293</v>
       </c>
     </row>
     <row r="69" spans="1:9">
       <c r="B69" s="5">
         <f t="shared" si="5"/>
-        <v>0.47061233885469206</v>
+        <v>0.3844398923190297</v>
       </c>
       <c r="C69" s="5">
         <f t="shared" si="6"/>
-        <v>0.52938766114530789</v>
+        <v>0.61556010768097025</v>
       </c>
       <c r="D69" s="5">
         <f t="shared" si="9"/>
@@ -1384,21 +1389,21 @@
       </c>
       <c r="F69" s="6">
         <f t="shared" si="7"/>
-        <v>0.34755515016257854</v>
+        <v>0.36024614552265033</v>
       </c>
       <c r="G69">
         <f t="shared" si="8"/>
-        <v>0.43158618115666919</v>
+        <v>0.41638197067279603</v>
       </c>
     </row>
     <row r="70" spans="1:9">
       <c r="B70" s="5">
         <f t="shared" si="5"/>
-        <v>0.46642594388759007</v>
+        <v>0.36865424647507272</v>
       </c>
       <c r="C70" s="5">
         <f t="shared" si="6"/>
-        <v>0.53357405611240993</v>
+        <v>0.63134575352492728</v>
       </c>
       <c r="D70" s="5">
         <f t="shared" si="9"/>
@@ -1410,21 +1415,21 @@
       </c>
       <c r="F70" s="6">
         <f t="shared" si="7"/>
-        <v>0.34817169896952149</v>
+        <v>0.36257096704293157</v>
       </c>
       <c r="G70">
         <f t="shared" si="8"/>
-        <v>0.43082192046037265</v>
+        <v>0.41371211055141843</v>
       </c>
     </row>
     <row r="71" spans="1:9">
       <c r="B71" s="5">
         <f t="shared" si="5"/>
-        <v>0.46224427223138398</v>
+        <v>0.35314492218309612</v>
       </c>
       <c r="C71" s="5">
         <f t="shared" si="6"/>
-        <v>0.53775572776861602</v>
+        <v>0.64685507781690388</v>
       </c>
       <c r="D71" s="5">
         <f t="shared" si="9"/>
@@ -1436,21 +1441,21 @@
       </c>
       <c r="F71" s="6">
         <f t="shared" si="7"/>
-        <v>0.34878755215368629</v>
+        <v>0.36485509347243783</v>
       </c>
       <c r="G71">
         <f t="shared" si="8"/>
-        <v>0.43006121942650488</v>
+        <v>0.411122121312338</v>
       </c>
     </row>
     <row r="72" spans="1:9">
       <c r="B72" s="5">
         <f t="shared" si="5"/>
-        <v>0.45806790581208973</v>
+        <v>2.4945865146310072E-15</v>
       </c>
       <c r="C72" s="5">
         <f t="shared" si="6"/>
-        <v>0.54193209418791022</v>
+        <v>0.99999999999999756</v>
       </c>
       <c r="D72" s="5">
         <f t="shared" si="9"/>
@@ -1462,11 +1467,11 @@
       </c>
       <c r="F72" s="6">
         <f t="shared" si="7"/>
-        <v>0.34940262401226796</v>
+        <v>0.41686429999999969</v>
       </c>
       <c r="G72">
         <f t="shared" si="8"/>
-        <v>0.42930415999031912</v>
+        <v>0.35982932575420851</v>
       </c>
       <c r="I72" t="s">
         <v>19</v>
@@ -1491,7 +1496,7 @@
       <c r="F74" s="5"/>
       <c r="I74">
         <f t="shared" si="11"/>
-        <v>-1.7651252146691498E-3</v>
+        <v>-6.4928061065077092E-3</v>
       </c>
     </row>
     <row r="75" spans="1:9">
@@ -1505,7 +1510,7 @@
       <c r="F75"/>
       <c r="I75">
         <f t="shared" si="11"/>
-        <v>-3.341466433864404E-3</v>
+        <v>-1.2784755301320228E-2</v>
       </c>
     </row>
     <row r="76" spans="1:9">
@@ -1532,7 +1537,7 @@
       </c>
       <c r="I76">
         <f t="shared" si="11"/>
-        <v>-4.9174239895139471E-3</v>
+        <v>-1.9052256394710587E-2</v>
       </c>
     </row>
     <row r="77" spans="1:9">
@@ -1563,17 +1568,17 @@
       </c>
       <c r="I77">
         <f t="shared" si="11"/>
-        <v>-6.4928061065077092E-3</v>
+        <v>-2.5283297089886581E-2</v>
       </c>
     </row>
     <row r="78" spans="1:9">
       <c r="B78" s="5">
         <f t="shared" si="12"/>
-        <v>0.49579701732317438</v>
+        <v>0.48319400653587524</v>
       </c>
       <c r="C78" s="5">
         <f t="shared" si="13"/>
-        <v>0.50420298267682562</v>
+        <v>0.5168059934641247</v>
       </c>
       <c r="D78" s="5">
         <v>-0.4166726</v>
@@ -1583,25 +1588,25 @@
       </c>
       <c r="F78" s="2">
         <f t="shared" si="14"/>
-        <v>-0.34246042516844777</v>
+        <v>-0.34060542455939646</v>
       </c>
       <c r="G78">
         <f t="shared" si="15"/>
-        <v>0.43800681473258912</v>
+        <v>0.44039228146186571</v>
       </c>
       <c r="I78">
         <f t="shared" si="11"/>
-        <v>-8.0674212626548614E-3</v>
+        <v>-3.1466119184320684E-2</v>
       </c>
     </row>
     <row r="79" spans="1:9">
       <c r="B79" s="5">
         <f t="shared" si="12"/>
-        <v>0.49159462857202485</v>
+        <v>0.46642594388759007</v>
       </c>
       <c r="C79" s="5">
         <f t="shared" si="13"/>
-        <v>0.50840537142797515</v>
+        <v>0.53357405611240993</v>
       </c>
       <c r="D79" s="5">
         <v>-0.4166726</v>
@@ -1611,25 +1616,25 @@
       </c>
       <c r="F79" s="2">
         <f t="shared" si="14"/>
-        <v>-0.3418418877550935</v>
+        <v>-0.33813738204557708</v>
       </c>
       <c r="G79">
         <f t="shared" si="15"/>
-        <v>0.43879935541271292</v>
+        <v>0.44360667576169288</v>
       </c>
       <c r="I79">
         <f t="shared" si="11"/>
-        <v>-9.6410782727475719E-3</v>
+        <v>-3.7589298316103192E-2</v>
       </c>
     </row>
     <row r="80" spans="1:9">
       <c r="B80" s="5">
         <f t="shared" si="12"/>
-        <v>0.4873934273365631</v>
+        <v>0.4497334012055223</v>
       </c>
       <c r="C80" s="5">
         <f t="shared" si="13"/>
-        <v>0.5126065726634369</v>
+        <v>0.5502665987944777</v>
       </c>
       <c r="D80" s="5">
         <v>-0.4166726</v>
@@ -1639,25 +1644,25 @@
       </c>
       <c r="F80" s="2">
         <f t="shared" si="14"/>
-        <v>-0.34122352512872944</v>
+        <v>-0.33568045509657729</v>
       </c>
       <c r="G80">
         <f t="shared" si="15"/>
-        <v>0.43959454420210692</v>
+        <v>0.44685354098690105</v>
       </c>
       <c r="I80">
         <f t="shared" si="11"/>
-        <v>-1.1213586372360529E-2</v>
+        <v>-4.3641819542204974E-2</v>
       </c>
     </row>
     <row r="81" spans="1:9">
       <c r="B81" s="5">
         <f t="shared" si="12"/>
-        <v>0.48319400653587524</v>
+        <v>0.4331532908282692</v>
       </c>
       <c r="C81" s="5">
         <f t="shared" si="13"/>
-        <v>0.5168059934641247</v>
+        <v>0.56684670917173086</v>
       </c>
       <c r="D81" s="5">
         <v>-0.4166726</v>
@@ -1667,25 +1672,25 @@
       </c>
       <c r="F81" s="2">
         <f t="shared" si="14"/>
-        <v>-0.34060542455939646</v>
+        <v>-0.33324007673246958</v>
       </c>
       <c r="G81">
         <f t="shared" si="15"/>
-        <v>0.44039228146186571</v>
+        <v>0.45012593164303694</v>
       </c>
       <c r="I81">
         <f t="shared" si="11"/>
-        <v>-1.2784755301320228E-2</v>
+        <v>-4.9613147822177406E-2</v>
       </c>
     </row>
     <row r="82" spans="1:9">
       <c r="B82" s="5">
         <f t="shared" si="12"/>
-        <v>0.47899695808366566</v>
+        <v>0.41672152596199674</v>
       </c>
       <c r="C82" s="5">
         <f t="shared" si="13"/>
-        <v>0.52100304191633429</v>
+        <v>0.58327847403800326</v>
       </c>
       <c r="D82" s="5">
         <v>-0.4166726</v>
@@ -1695,25 +1700,25 @@
       </c>
       <c r="F82" s="2">
         <f t="shared" si="14"/>
-        <v>-0.33998767316915629</v>
+        <v>-0.33082153291392102</v>
       </c>
       <c r="G82">
         <f t="shared" si="15"/>
-        <v>0.44119246619088309</v>
+        <v>0.45341667659532198</v>
       </c>
       <c r="I82">
         <f t="shared" si="11"/>
-        <v>-1.4354395386779517E-2</v>
+        <v>-5.5493292559703922E-2</v>
       </c>
     </row>
     <row r="83" spans="1:9">
       <c r="B83" s="5">
         <f t="shared" si="12"/>
-        <v>0.47480287255500653</v>
+        <v>0.40047271707730309</v>
       </c>
       <c r="C83" s="5">
         <f t="shared" si="13"/>
-        <v>0.52519712744499347</v>
+        <v>0.59952728292269697</v>
       </c>
       <c r="D83" s="5">
         <v>-0.4166726</v>
@@ -1723,25 +1728,25 @@
       </c>
       <c r="F83" s="2">
         <f t="shared" si="14"/>
-        <v>-0.33937035788304104</v>
+        <v>-0.32842991785572873</v>
       </c>
       <c r="G83">
         <f t="shared" si="15"/>
-        <v>0.44199499607356774</v>
+        <v>0.45671844081479612</v>
       </c>
       <c r="I83">
         <f t="shared" si="11"/>
-        <v>-1.5922317625830018E-2</v>
+        <v>-0.19678689292917068</v>
       </c>
     </row>
     <row r="84" spans="1:9">
       <c r="B84" s="5">
         <f t="shared" si="12"/>
-        <v>0.47061233885469206</v>
+        <v>0.3844398923190297</v>
       </c>
       <c r="C84" s="5">
         <f t="shared" si="13"/>
-        <v>0.52938766114530789</v>
+        <v>0.61556010768097025</v>
       </c>
       <c r="D84" s="5">
         <v>-0.4166726</v>
@@ -1751,21 +1756,21 @@
       </c>
       <c r="F84" s="2">
         <f t="shared" si="14"/>
-        <v>-0.33875356538023943</v>
+        <v>-0.32607009287475025</v>
       </c>
       <c r="G84">
         <f t="shared" si="15"/>
-        <v>0.44279976752902972</v>
+        <v>0.460023790215001</v>
       </c>
     </row>
     <row r="85" spans="1:9">
       <c r="B85" s="5">
         <f t="shared" si="12"/>
-        <v>0.46642594388759007</v>
+        <v>0.36865424647507272</v>
       </c>
       <c r="C85" s="5">
         <f t="shared" si="13"/>
-        <v>0.53357405611240993</v>
+        <v>0.63134575352492728</v>
       </c>
       <c r="D85" s="5">
         <v>-0.4166726</v>
@@ -1775,21 +1780,21 @@
       </c>
       <c r="F85" s="2">
         <f t="shared" si="14"/>
-        <v>-0.33813738204557708</v>
+        <v>-0.32374664944135118</v>
       </c>
       <c r="G85">
         <f t="shared" si="15"/>
-        <v>0.44360667576169288</v>
+        <v>0.46332525837359584</v>
       </c>
     </row>
     <row r="86" spans="1:9">
       <c r="B86" s="5">
         <f t="shared" si="12"/>
-        <v>0.46224427223138398</v>
+        <v>0.35314492218309612</v>
       </c>
       <c r="C86" s="5">
         <f t="shared" si="13"/>
-        <v>0.53775572776861602</v>
+        <v>0.64685507781690388</v>
       </c>
       <c r="D86" s="5">
         <v>-0.4166726</v>
@@ -1799,21 +1804,21 @@
       </c>
       <c r="F86" s="2">
         <f t="shared" si="14"/>
-        <v>-0.3375218939213479</v>
+        <v>-0.32146387697585554</v>
       </c>
       <c r="G86">
         <f t="shared" si="15"/>
-        <v>0.4444156148132844</v>
+        <v>0.46661541387204192</v>
       </c>
     </row>
     <row r="87" spans="1:9">
       <c r="B87" s="5">
         <f t="shared" si="12"/>
-        <v>0.45806790581208973</v>
+        <v>2.4945865146310072E-15</v>
       </c>
       <c r="C87" s="5">
         <f t="shared" si="13"/>
-        <v>0.54193209418791022</v>
+        <v>0.99999999999999756</v>
       </c>
       <c r="D87" s="5">
         <v>-0.4166726</v>
@@ -1823,11 +1828,11 @@
       </c>
       <c r="F87" s="2">
         <f t="shared" si="14"/>
-        <v>-0.33690718665955466</v>
+        <v>-0.26948550000000038</v>
       </c>
       <c r="G87">
         <f t="shared" si="15"/>
-        <v>0.44522647761614914</v>
+        <v>0.55661621868337918</v>
       </c>
     </row>
     <row r="90" spans="1:9">
@@ -1835,7 +1840,7 @@
     </row>
     <row r="93" spans="1:9">
       <c r="A93" t="s">
-        <v>21</v>
+        <v>24</v>
       </c>
     </row>
     <row r="94" spans="1:9">
@@ -1874,258 +1879,258 @@
         <v>0.5</v>
       </c>
       <c r="D95" s="5">
-        <v>0.33046300000000001</v>
+        <v>0.2411276</v>
       </c>
       <c r="E95" s="5">
         <v>0.58988229999999997</v>
       </c>
       <c r="F95" s="2">
         <f t="shared" ref="F95:F105" si="18">B95*D95+C95*E95</f>
-        <v>0.46017264999999996</v>
+        <v>0.41550494999999998</v>
       </c>
       <c r="G95">
         <f t="shared" ref="G95:G105" si="19">0.0765/F95</f>
-        <v>0.16624195288442284</v>
+        <v>0.18411333005780076</v>
       </c>
     </row>
     <row r="96" spans="1:9">
       <c r="B96" s="5">
         <f t="shared" si="16"/>
-        <v>0.49579701732317438</v>
+        <v>0.48319400653587524</v>
       </c>
       <c r="C96" s="5">
         <f t="shared" si="17"/>
-        <v>0.50420298267682562</v>
+        <v>0.5168059934641247</v>
       </c>
       <c r="D96" s="5">
-        <v>0.33046300000000001</v>
+        <v>0.2411276</v>
       </c>
       <c r="E96" s="5">
         <v>0.58988229999999997</v>
       </c>
       <c r="F96" s="2">
         <f t="shared" si="18"/>
-        <v>0.46126298482393424</v>
+        <v>0.42136611920878275</v>
       </c>
       <c r="G96">
         <f t="shared" si="19"/>
-        <v>0.1658489896586875</v>
+        <v>0.18155232827842763</v>
       </c>
     </row>
     <row r="97" spans="1:12">
       <c r="B97" s="5">
         <f t="shared" si="16"/>
-        <v>0.49159462857202485</v>
+        <v>0.46642594388759007</v>
       </c>
       <c r="C97" s="5">
         <f t="shared" si="17"/>
-        <v>0.50840537142797515</v>
+        <v>0.53357405611240993</v>
       </c>
       <c r="D97" s="5">
-        <v>0.33046300000000001</v>
+        <v>0.2411276</v>
       </c>
       <c r="E97" s="5">
         <v>0.58988229999999997</v>
       </c>
       <c r="F97" s="2">
         <f t="shared" si="18"/>
-        <v>0.46235316557208533</v>
+        <v>0.42721405986726668</v>
       </c>
       <c r="G97">
         <f t="shared" si="19"/>
-        <v>0.16545793496480973</v>
+        <v>0.1790671403084631</v>
       </c>
     </row>
     <row r="98" spans="1:12">
       <c r="B98" s="5">
         <f t="shared" si="16"/>
-        <v>0.4873934273365631</v>
+        <v>0.4497334012055223</v>
       </c>
       <c r="C98" s="5">
         <f t="shared" si="17"/>
-        <v>0.5126065726634369</v>
+        <v>0.5502665987944777</v>
       </c>
       <c r="D98" s="5">
-        <v>0.33046300000000001</v>
+        <v>0.2411276</v>
       </c>
       <c r="E98" s="5">
         <v>0.58988229999999997</v>
       </c>
       <c r="F98" s="2">
         <f t="shared" si="18"/>
-        <v>0.4634430382557479</v>
+        <v>0.43303566258258841</v>
       </c>
       <c r="G98">
         <f t="shared" si="19"/>
-        <v>0.16506882979172943</v>
+        <v>0.17665981490706886</v>
       </c>
     </row>
     <row r="99" spans="1:12">
       <c r="B99" s="5">
         <f t="shared" si="16"/>
-        <v>0.48319400653587524</v>
+        <v>0.4331532908282692</v>
       </c>
       <c r="C99" s="5">
         <f t="shared" si="17"/>
-        <v>0.5168059934641247</v>
+        <v>0.56684670917173086</v>
       </c>
       <c r="D99" s="5">
-        <v>0.33046300000000001</v>
+        <v>0.2411276</v>
       </c>
       <c r="E99" s="5">
         <v>0.58988229999999997</v>
       </c>
       <c r="F99" s="2">
         <f t="shared" si="18"/>
-        <v>0.46453244906026775</v>
+        <v>0.43881805400317425</v>
       </c>
       <c r="G99">
         <f t="shared" si="19"/>
-        <v>0.16468171417251198</v>
+        <v>0.17433193393507604</v>
       </c>
     </row>
     <row r="100" spans="1:12">
       <c r="B100" s="5">
         <f t="shared" si="16"/>
-        <v>0.47899695808366566</v>
+        <v>0.41672152596199674</v>
       </c>
       <c r="C100" s="5">
         <f t="shared" si="17"/>
-        <v>0.52100304191633429</v>
+        <v>0.58327847403800326</v>
       </c>
       <c r="D100" s="5">
-        <v>0.33046300000000001</v>
+        <v>0.2411276</v>
       </c>
       <c r="E100" s="5">
         <v>0.58988229999999997</v>
       </c>
       <c r="F100" s="2">
         <f t="shared" si="18"/>
-        <v>0.46562124443180608</v>
+        <v>0.44454870922958156</v>
       </c>
       <c r="G100">
         <f t="shared" si="19"/>
-        <v>0.16429662717248295</v>
+        <v>0.17208462967438859</v>
       </c>
     </row>
     <row r="101" spans="1:12">
       <c r="B101" s="5">
         <f t="shared" si="16"/>
-        <v>0.47480287255500653</v>
+        <v>0.40047271707730309</v>
       </c>
       <c r="C101" s="5">
         <f t="shared" si="17"/>
-        <v>0.52519712744499347</v>
+        <v>0.59952728292269697</v>
       </c>
       <c r="D101" s="5">
-        <v>0.33046300000000001</v>
+        <v>0.2411276</v>
       </c>
       <c r="E101" s="5">
         <v>0.58988229999999997</v>
       </c>
       <c r="F101" s="2">
         <f t="shared" si="18"/>
-        <v>0.46670927116379102</v>
+        <v>0.45021555769752031</v>
       </c>
       <c r="G101">
         <f t="shared" si="19"/>
-        <v>0.16391360687830095</v>
+        <v>0.1699186060811273</v>
       </c>
     </row>
     <row r="102" spans="1:12">
       <c r="B102" s="5">
         <f t="shared" si="16"/>
-        <v>0.47061233885469206</v>
+        <v>0.3844398923190297</v>
       </c>
       <c r="C102" s="5">
         <f t="shared" si="17"/>
-        <v>0.52938766114530789</v>
+        <v>0.61556010768097025</v>
       </c>
       <c r="D102" s="5">
-        <v>0.33046300000000001</v>
+        <v>0.2411276</v>
       </c>
       <c r="E102" s="5">
         <v>0.58988229999999997</v>
       </c>
       <c r="F102" s="2">
         <f t="shared" si="18"/>
-        <v>0.46779637648295297</v>
+        <v>0.45580708068624443</v>
       </c>
       <c r="G102">
         <f t="shared" si="19"/>
-        <v>0.16353269038796786</v>
+        <v>0.16783416327105918</v>
       </c>
     </row>
     <row r="103" spans="1:12">
       <c r="B103" s="5">
         <f t="shared" si="16"/>
-        <v>0.46642594388759007</v>
+        <v>0.36865424647507272</v>
       </c>
       <c r="C103" s="5">
         <f t="shared" si="17"/>
-        <v>0.53357405611240993</v>
+        <v>0.63134575352492728</v>
       </c>
       <c r="D103" s="5">
-        <v>0.33046300000000001</v>
+        <v>0.2411276</v>
       </c>
       <c r="E103" s="5">
         <v>0.58988229999999997</v>
       </c>
       <c r="F103" s="2">
         <f t="shared" si="18"/>
-        <v>0.46888240813484211</v>
+        <v>0.46131239886685993</v>
       </c>
       <c r="G103">
         <f t="shared" si="19"/>
-        <v>0.16315391380177346</v>
+        <v>0.16583122454091848</v>
       </c>
     </row>
     <row r="104" spans="1:12">
       <c r="B104" s="5">
         <f t="shared" si="16"/>
-        <v>0.46224427223138398</v>
+        <v>0.35314492218309612</v>
       </c>
       <c r="C104" s="5">
         <f t="shared" si="17"/>
-        <v>0.53775572776861602</v>
+        <v>0.64685507781690388</v>
       </c>
       <c r="D104" s="5">
-        <v>0.33046300000000001</v>
+        <v>0.2411276</v>
       </c>
       <c r="E104" s="5">
         <v>0.58988229999999997</v>
       </c>
       <c r="F104" s="2">
         <f t="shared" si="18"/>
-        <v>0.46996721446872491</v>
+        <v>0.46672134860751097</v>
       </c>
       <c r="G104">
         <f t="shared" si="19"/>
-        <v>0.16277731221417122</v>
+        <v>0.16390936525239738</v>
       </c>
     </row>
     <row r="105" spans="1:12">
       <c r="B105" s="5">
         <f t="shared" si="16"/>
-        <v>0.45806790581208973</v>
+        <v>2.4945865146310072E-15</v>
       </c>
       <c r="C105" s="5">
         <f t="shared" si="17"/>
-        <v>0.54193209418791022</v>
+        <v>0.99999999999999756</v>
       </c>
       <c r="D105" s="5">
-        <v>0.33046300000000001</v>
+        <v>0.2411276</v>
       </c>
       <c r="E105" s="5">
         <v>0.58988229999999997</v>
       </c>
       <c r="F105" s="2">
         <f t="shared" si="18"/>
-        <v>0.47105064452176171</v>
+        <v>0.58988229999999908</v>
       </c>
       <c r="G105">
         <f t="shared" si="19"/>
-        <v>0.16240291970657911</v>
+        <v>0.129686888384344</v>
       </c>
     </row>
     <row r="106" spans="1:12">
@@ -2134,20 +2139,20 @@
         <v>19</v>
       </c>
       <c r="J106" t="s">
+        <v>21</v>
+      </c>
+      <c r="K106" t="s">
         <v>22</v>
       </c>
-      <c r="K106" t="s">
+      <c r="L106" t="s">
         <v>23</v>
-      </c>
-      <c r="L106" t="s">
-        <v>24</v>
       </c>
     </row>
     <row r="107" spans="1:12">
       <c r="B107" s="5"/>
       <c r="I107" s="5">
         <f t="shared" ref="I107:I117" si="20">G95-G110</f>
-        <v>-7.510373414268412E-5</v>
+        <v>-4.6345338838566508E-3</v>
       </c>
       <c r="J107" s="8">
         <f t="shared" ref="J107:J117" si="21">I107-I$107</f>
@@ -2168,19 +2173,19 @@
       </c>
       <c r="I108" s="5">
         <f t="shared" si="20"/>
-        <v>-8.6320761755037667E-4</v>
+        <v>-4.6843951695748065E-3</v>
       </c>
       <c r="J108" s="8">
         <f t="shared" si="21"/>
-        <v>-7.8810388340769255E-4</v>
+        <v>-4.9861285718155735E-5</v>
       </c>
       <c r="K108">
         <f t="shared" si="22"/>
-        <v>-1.9702597085192314E-3</v>
+        <v>-1.2465321429538934E-4</v>
       </c>
       <c r="L108">
         <f t="shared" si="23"/>
-        <v>-5.130884657602165E-3</v>
+        <v>-3.2461774556090975E-4</v>
       </c>
     </row>
     <row r="109" spans="1:12">
@@ -2207,19 +2212,19 @@
       </c>
       <c r="I109" s="5">
         <f t="shared" si="20"/>
-        <v>-1.6512287756165478E-3</v>
+        <v>-4.729829300098215E-3</v>
       </c>
       <c r="J109" s="8">
         <f t="shared" si="21"/>
-        <v>-1.5761250414738637E-3</v>
+        <v>-9.5295416241564235E-5</v>
       </c>
       <c r="K109">
         <f t="shared" si="22"/>
-        <v>-3.9403126036846592E-3</v>
+        <v>-2.3823854060391059E-4</v>
       </c>
       <c r="L109">
         <f t="shared" si="23"/>
-        <v>-1.0261230738762133E-2</v>
+        <v>-6.2041286615601712E-4</v>
       </c>
     </row>
     <row r="110" spans="1:12">
@@ -2235,387 +2240,387 @@
         <v>0.5</v>
       </c>
       <c r="D110" s="5">
-        <v>-0.5896593</v>
+        <v>-0.2427137</v>
       </c>
       <c r="E110" s="5">
-        <v>-0.33027040000000002</v>
+        <v>-0.56789149999999999</v>
       </c>
       <c r="F110" s="2">
         <f t="shared" ref="F110:F120" si="26">B110*D110+C110*E110</f>
-        <v>-0.45996484999999998</v>
+        <v>-0.40530260000000001</v>
       </c>
       <c r="G110">
         <f t="shared" ref="G110:G120" si="27">-0.0765/F110</f>
-        <v>0.16631705661856552</v>
+        <v>0.18874786394165741</v>
       </c>
       <c r="I110" s="5">
         <f t="shared" si="20"/>
-        <v>-2.4390824175049564E-3</v>
+        <v>-4.7710634034219546E-3</v>
       </c>
       <c r="J110" s="8">
         <f t="shared" si="21"/>
-        <v>-2.3639786833622722E-3</v>
+        <v>-1.3652951956530379E-4</v>
       </c>
       <c r="K110">
         <f t="shared" si="22"/>
-        <v>-5.9099467084056806E-3</v>
+        <v>-3.4132379891325948E-4</v>
       </c>
       <c r="L110">
         <f t="shared" si="23"/>
-        <v>-1.539048621980646E-2</v>
+        <v>-8.8886405966994656E-4</v>
       </c>
     </row>
     <row r="111" spans="1:12">
       <c r="B111" s="5">
         <f t="shared" si="24"/>
-        <v>0.49579701732317438</v>
+        <v>0.48319400653587524</v>
       </c>
       <c r="C111" s="5">
         <f t="shared" si="25"/>
-        <v>0.50420298267682562</v>
+        <v>0.5168059934641247</v>
       </c>
       <c r="D111" s="5">
-        <v>-0.5896593</v>
+        <v>-0.2427137</v>
       </c>
       <c r="E111" s="5">
-        <v>-0.33027040000000002</v>
+        <v>-0.56789149999999999</v>
       </c>
       <c r="F111" s="2">
         <f t="shared" si="26"/>
-        <v>-0.45887464294673919</v>
+        <v>-0.41076753598147847</v>
       </c>
       <c r="G111">
         <f t="shared" si="27"/>
-        <v>0.16671219727623787</v>
+        <v>0.18623672344800243</v>
       </c>
       <c r="I111" s="5">
         <f t="shared" si="20"/>
-        <v>-3.2266838082411486E-3</v>
+        <v>-4.8083336372191365E-3</v>
       </c>
       <c r="J111" s="8">
         <f t="shared" si="21"/>
-        <v>-3.1515800740984645E-3</v>
+        <v>-1.7379975336248576E-4</v>
       </c>
       <c r="K111">
         <f t="shared" si="22"/>
-        <v>-7.8789501852461613E-3</v>
+        <v>-4.3449938340621441E-4</v>
       </c>
       <c r="L111">
         <f t="shared" si="23"/>
-        <v>-2.0518099440745213E-2</v>
+        <v>-1.1315088109536834E-3</v>
       </c>
     </row>
     <row r="112" spans="1:12">
       <c r="B112" s="5">
         <f t="shared" si="24"/>
-        <v>0.49159462857202485</v>
+        <v>0.46642594388759007</v>
       </c>
       <c r="C112" s="5">
         <f t="shared" si="25"/>
-        <v>0.50840537142797515</v>
+        <v>0.53357405611240993</v>
       </c>
       <c r="D112" s="5">
-        <v>-0.5896593</v>
+        <v>-0.2427137</v>
       </c>
       <c r="E112" s="5">
-        <v>-0.33027040000000002</v>
+        <v>-0.56789149999999999</v>
       </c>
       <c r="F112" s="2">
         <f t="shared" si="26"/>
-        <v>-0.45778458995120608</v>
+        <v>-0.41622013770371002</v>
       </c>
       <c r="G112">
         <f t="shared" si="27"/>
-        <v>0.16710916374042628</v>
+        <v>0.18379696960856132</v>
       </c>
       <c r="I112" s="5">
         <f t="shared" si="20"/>
-        <v>-4.0139482971032481E-3</v>
+        <v>-4.8418816613403359E-3</v>
       </c>
       <c r="J112" s="8">
         <f t="shared" si="21"/>
-        <v>-3.938844562960564E-3</v>
+        <v>-2.0734777748368516E-4</v>
       </c>
       <c r="K112">
         <f t="shared" si="22"/>
-        <v>-9.8471114074014099E-3</v>
+        <v>-5.183694437092129E-4</v>
       </c>
       <c r="L112">
         <f t="shared" si="23"/>
-        <v>-2.5643519290107837E-2</v>
+        <v>-1.3499204263260752E-3</v>
       </c>
     </row>
     <row r="113" spans="2:12">
       <c r="B113" s="5">
         <f t="shared" si="24"/>
-        <v>0.4873934273365631</v>
+        <v>0.4497334012055223</v>
       </c>
       <c r="C113" s="5">
         <f t="shared" si="25"/>
-        <v>0.5126065726634369</v>
+        <v>0.5502665987944777</v>
       </c>
       <c r="D113" s="5">
-        <v>-0.5896593</v>
+        <v>-0.2427137</v>
       </c>
       <c r="E113" s="5">
-        <v>-0.33027040000000002</v>
+        <v>-0.56789149999999999</v>
       </c>
       <c r="F113" s="2">
         <f t="shared" si="26"/>
-        <v>-0.45669484498406099</v>
+        <v>-0.42164818200947091</v>
       </c>
       <c r="G113">
         <f t="shared" si="27"/>
-        <v>0.16750791220923439</v>
+        <v>0.18143087831049082</v>
       </c>
       <c r="I113" s="5">
         <f t="shared" si="20"/>
-        <v>-4.8007913459895968E-3</v>
+        <v>-4.8719514015262977E-3</v>
       </c>
       <c r="J113" s="8">
         <f t="shared" si="21"/>
-        <v>-4.7256876118469127E-3</v>
+        <v>-2.3741751766964692E-4</v>
       </c>
       <c r="K113">
         <f t="shared" si="22"/>
-        <v>-1.1814219029617282E-2</v>
+        <v>-5.9354379417411729E-4</v>
       </c>
       <c r="L113">
         <f t="shared" si="23"/>
-        <v>-3.0766195389628336E-2</v>
+        <v>-1.5456869639950972E-3</v>
       </c>
     </row>
     <row r="114" spans="2:12">
       <c r="B114" s="5">
         <f t="shared" si="24"/>
-        <v>0.48319400653587524</v>
+        <v>0.4331532908282692</v>
       </c>
       <c r="C114" s="5">
         <f t="shared" si="25"/>
-        <v>0.5168059934641247</v>
+        <v>0.56684670917173086</v>
       </c>
       <c r="D114" s="5">
-        <v>-0.5896593</v>
+        <v>-0.2427137</v>
       </c>
       <c r="E114" s="5">
-        <v>-0.33027040000000002</v>
+        <v>-0.56789149999999999</v>
       </c>
       <c r="F114" s="2">
         <f t="shared" si="26"/>
-        <v>-0.45560556184193346</v>
+        <v>-0.4270396658257033</v>
       </c>
       <c r="G114">
         <f t="shared" si="27"/>
-        <v>0.16790839798075313</v>
+        <v>0.17914026757229518</v>
       </c>
       <c r="I114" s="5">
         <f t="shared" si="20"/>
-        <v>-5.5871285577545893E-3</v>
+        <v>-4.8987861386075859E-3</v>
       </c>
       <c r="J114" s="8">
         <f t="shared" si="21"/>
-        <v>-5.5120248236119052E-3</v>
+        <v>-2.6425225475093517E-4</v>
       </c>
       <c r="K114">
         <f t="shared" si="22"/>
-        <v>-1.3780062059029763E-2</v>
+        <v>-6.6063063687733792E-4</v>
       </c>
       <c r="L114">
         <f t="shared" si="23"/>
-        <v>-3.5885578278723337E-2</v>
+        <v>-1.7203922835347342E-3</v>
       </c>
     </row>
     <row r="115" spans="2:12">
       <c r="B115" s="5">
         <f t="shared" si="24"/>
-        <v>0.47899695808366566</v>
+        <v>0.41672152596199674</v>
       </c>
       <c r="C115" s="5">
         <f t="shared" si="25"/>
-        <v>0.52100304191633429</v>
+        <v>0.58327847403800326</v>
       </c>
       <c r="D115" s="5">
-        <v>-0.5896593</v>
+        <v>-0.2427137</v>
       </c>
       <c r="E115" s="5">
-        <v>-0.33027040000000002</v>
+        <v>-0.56789149999999999</v>
       </c>
       <c r="F115" s="2">
         <f t="shared" si="26"/>
-        <v>-0.45451689406066814</v>
+        <v>-0.43238291097503501</v>
       </c>
       <c r="G115">
         <f t="shared" si="27"/>
-        <v>0.16831057546958619</v>
+        <v>0.17692651133572893</v>
       </c>
       <c r="I115" s="5">
         <f t="shared" si="20"/>
-        <v>-6.3728757045048712E-3</v>
+        <v>-4.9226259441777775E-3</v>
       </c>
       <c r="J115" s="8">
         <f t="shared" si="21"/>
-        <v>-6.2977719703621871E-3</v>
+        <v>-2.8809206032112677E-4</v>
       </c>
       <c r="K115">
         <f t="shared" si="22"/>
-        <v>-1.5744429925905468E-2</v>
+        <v>-7.2023015080281694E-4</v>
       </c>
       <c r="L115">
         <f t="shared" si="23"/>
-        <v>-4.1001119598712152E-2</v>
+        <v>-1.8755993510490023E-3</v>
       </c>
     </row>
     <row r="116" spans="2:12">
       <c r="B116" s="5">
         <f t="shared" si="24"/>
-        <v>0.47480287255500653</v>
+        <v>0.40047271707730309</v>
       </c>
       <c r="C116" s="5">
         <f t="shared" si="25"/>
-        <v>0.52519712744499347</v>
+        <v>0.59952728292269697</v>
       </c>
       <c r="D116" s="5">
-        <v>-0.5896593</v>
+        <v>-0.2427137</v>
       </c>
       <c r="E116" s="5">
-        <v>-0.33027040000000002</v>
+        <v>-0.56789149999999999</v>
       </c>
       <c r="F116" s="2">
         <f t="shared" si="26"/>
-        <v>-0.45342899482888332</v>
+        <v>-0.43766666290078021</v>
       </c>
       <c r="G116">
         <f t="shared" si="27"/>
-        <v>0.16871439822429055</v>
+        <v>0.1747905574826536</v>
       </c>
       <c r="I116" s="5">
         <f t="shared" si="20"/>
-        <v>-7.1579487558466326E-3</v>
+        <v>-4.9437054716393869E-3</v>
       </c>
       <c r="J116" s="8">
         <f t="shared" si="21"/>
-        <v>-7.0828450217039485E-3</v>
+        <v>-3.0917158778273612E-4</v>
       </c>
       <c r="K116">
         <f t="shared" si="22"/>
-        <v>-1.7707112554259871E-2</v>
+        <v>-7.7292896945684031E-4</v>
       </c>
       <c r="L116">
         <f t="shared" si="23"/>
-        <v>-4.6112272276718415E-2</v>
+        <v>-2.0128358579605218E-3</v>
       </c>
     </row>
     <row r="117" spans="2:12">
       <c r="B117" s="5">
         <f t="shared" si="24"/>
-        <v>0.47061233885469206</v>
+        <v>0.3844398923190297</v>
       </c>
       <c r="C117" s="5">
         <f t="shared" si="25"/>
-        <v>0.52938766114530789</v>
+        <v>0.61556010768097025</v>
       </c>
       <c r="D117" s="5">
-        <v>-0.5896593</v>
+        <v>-0.2427137</v>
       </c>
       <c r="E117" s="5">
-        <v>-0.33027040000000002</v>
+        <v>-0.56789149999999999</v>
       </c>
       <c r="F117" s="2">
         <f t="shared" si="26"/>
-        <v>-0.45234201690194581</v>
+        <v>-0.44288018158346099</v>
       </c>
       <c r="G117">
         <f t="shared" si="27"/>
-        <v>0.16911981894572245</v>
+        <v>0.17273294940966677</v>
       </c>
       <c r="I117" s="5">
         <f t="shared" si="20"/>
-        <v>-7.942263907075725E-3</v>
+        <v>-5.0219424398541268E-3</v>
       </c>
       <c r="J117" s="8">
         <f t="shared" si="21"/>
-        <v>-7.8671601729330409E-3</v>
+        <v>-3.8740855599747603E-4</v>
       </c>
       <c r="K117">
         <f t="shared" si="22"/>
-        <v>-1.9667900432332602E-2</v>
+        <v>-9.6852138999369008E-4</v>
       </c>
       <c r="L117">
-        <f t="shared" si="23"/>
-        <v>-5.1218490709199482E-2</v>
+        <f>K117/0.192/2</f>
+        <v>-2.5221911197752345E-3</v>
       </c>
     </row>
     <row r="118" spans="2:12">
       <c r="B118" s="5">
         <f t="shared" si="24"/>
-        <v>0.46642594388759007</v>
+        <v>0.36865424647507272</v>
       </c>
       <c r="C118" s="5">
         <f t="shared" si="25"/>
-        <v>0.53357405611240993</v>
+        <v>0.63134575352492728</v>
       </c>
       <c r="D118" s="5">
-        <v>-0.5896593</v>
+        <v>-0.2427137</v>
       </c>
       <c r="E118" s="5">
-        <v>-0.33027040000000002</v>
+        <v>-0.56789149999999999</v>
       </c>
       <c r="F118" s="2">
         <f t="shared" si="26"/>
-        <v>-0.45125611251646369</v>
+        <v>-0.44801332317057807</v>
       </c>
       <c r="G118">
         <f t="shared" si="27"/>
-        <v>0.16952678950627834</v>
+        <v>0.17075385048509625</v>
       </c>
       <c r="I118" s="5"/>
     </row>
     <row r="119" spans="2:12">
       <c r="B119" s="5">
         <f t="shared" si="24"/>
-        <v>0.46224427223138398</v>
+        <v>0.35314492218309612</v>
       </c>
       <c r="C119" s="5">
         <f t="shared" si="25"/>
-        <v>0.53775572776861602</v>
+        <v>0.64685507781690388</v>
       </c>
       <c r="D119" s="5">
-        <v>-0.5896593</v>
+        <v>-0.2427137</v>
       </c>
       <c r="E119" s="5">
-        <v>-0.33027040000000002</v>
+        <v>-0.56789149999999999</v>
       </c>
       <c r="F119" s="2">
         <f t="shared" si="26"/>
-        <v>-0.45017143330539922</v>
+        <v>-0.45305661112332962</v>
       </c>
       <c r="G119">
         <f t="shared" si="27"/>
-        <v>0.16993526097001785</v>
+        <v>0.16885307072403677</v>
       </c>
     </row>
     <row r="120" spans="2:12">
       <c r="B120" s="5">
         <f t="shared" si="24"/>
-        <v>0.45806790581208973</v>
+        <v>2.4945865146310072E-15</v>
       </c>
       <c r="C120" s="5">
         <f t="shared" si="25"/>
-        <v>0.54193209418791022</v>
+        <v>0.99999999999999756</v>
       </c>
       <c r="D120" s="5">
-        <v>-0.5896593</v>
+        <v>-0.2427137</v>
       </c>
       <c r="E120" s="5">
-        <v>-0.33027040000000002</v>
+        <v>-0.56789149999999999</v>
       </c>
       <c r="F120" s="2">
         <f t="shared" si="26"/>
-        <v>-0.44908813021390159</v>
+        <v>-0.56789149999999922</v>
       </c>
       <c r="G120">
         <f t="shared" si="27"/>
-        <v>0.17034518361365483</v>
+        <v>0.13470883082419813</v>
       </c>
     </row>
     <row r="121" spans="2:12">

</xml_diff>